<commit_message>
update  no annd  key
</commit_message>
<xml_diff>
--- a/candidates_hiring.xlsx
+++ b/candidates_hiring.xlsx
@@ -627,7 +627,7 @@
         <v>Interview Scheduled</v>
       </c>
       <c r="H5" t="str">
-        <v>20-Aug-2026, 2:00 pm</v>
+        <v>22-Aug-2026, 11:00 am</v>
       </c>
       <c r="I5" t="str">
         <v/>
@@ -639,16 +639,16 @@
         <v>NO</v>
       </c>
       <c r="L5" t="str">
-        <v>YES</v>
+        <v>NO</v>
       </c>
       <c r="M5" t="str">
         <v>20-Aug-2026, 2:12 pm</v>
       </c>
       <c r="N5" t="str">
-        <v>Selected</v>
+        <v>Thank you</v>
       </c>
       <c r="O5" t="str">
-        <v>Auto-scheduled via WhatsApp AI: "Today 5 pm coming"</v>
+        <v>Auto-scheduled via WhatsApp AI: "Me kal interview Dene a nhi ska tha to kya mera interview resedule kr skte ho"</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add to pdf save data
</commit_message>
<xml_diff>
--- a/candidates_hiring.xlsx
+++ b/candidates_hiring.xlsx
@@ -627,7 +627,7 @@
         <v>Interview Scheduled</v>
       </c>
       <c r="H5" t="str">
-        <v>22-Aug-2026, 11:00 am</v>
+        <v>21-Aug-2026, 1:00 pm</v>
       </c>
       <c r="I5" t="str">
         <v/>
@@ -645,10 +645,10 @@
         <v>20-Aug-2026, 2:12 pm</v>
       </c>
       <c r="N5" t="str">
-        <v>manisha meena.pdf</v>
+        <v>Apply</v>
       </c>
       <c r="O5" t="str">
-        <v>Auto-scheduled via WhatsApp AI: "Me kal interview Dene a nhi ska tha to kya mera interview resedule kr skte ho"</v>
+        <v>Auto-scheduled via WhatsApp AI: "Arjun_Meena Backen Resume (1).pdf"</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix auto reply flow, sanitize candidate names, handle not interested intent, and improve unread badge UI
</commit_message>
<xml_diff>
--- a/candidates_hiring.xlsx
+++ b/candidates_hiring.xlsx
@@ -589,7 +589,7 @@
         <v/>
       </c>
       <c r="H4" t="str">
-        <v>Applied</v>
+        <v>Resume Pending</v>
       </c>
       <c r="I4" t="str">
         <v>Not Scheduled</v>
@@ -601,7 +601,7 @@
         <v>Indore</v>
       </c>
       <c r="L4" t="str">
-        <v>NO</v>
+        <v>YES</v>
       </c>
       <c r="M4" t="str">
         <v>NO</v>
@@ -690,7 +690,7 @@
         <v/>
       </c>
       <c r="H6" t="str">
-        <v>Applied</v>
+        <v>Resume Pending</v>
       </c>
       <c r="I6" t="str">
         <v>Not Scheduled</v>
@@ -702,7 +702,7 @@
         <v>Indore</v>
       </c>
       <c r="L6" t="str">
-        <v>NO</v>
+        <v>YES</v>
       </c>
       <c r="M6" t="str">
         <v>NO</v>

</xml_diff>

<commit_message>
update Ai chat bot
</commit_message>
<xml_diff>
--- a/candidates_hiring.xlsx
+++ b/candidates_hiring.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:P13"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -471,28 +471,28 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Bhumi</v>
+        <v>Arjun Meena</v>
       </c>
       <c r="C2" t="str">
-        <v>+919302051795</v>
+        <v>+918357977322</v>
       </c>
       <c r="D2" t="str">
-        <v>Graphic Designer</v>
+        <v>SEO &amp; AEO Expert</v>
       </c>
       <c r="E2" t="str">
         <v>In-Person (Indore Office)</v>
       </c>
       <c r="F2" t="str">
-        <v>PENDING</v>
+        <v>YES</v>
       </c>
       <c r="G2" t="str">
         <v/>
       </c>
       <c r="H2" t="str">
-        <v>Applied</v>
+        <v>Interview Scheduled</v>
       </c>
       <c r="I2" t="str">
-        <v>Not Scheduled</v>
+        <v>08-Sept-2026, 11:00 am</v>
       </c>
       <c r="J2" t="str">
         <v>Experienced (Full-Time)</v>
@@ -507,13 +507,13 @@
         <v>NO</v>
       </c>
       <c r="N2" t="str">
-        <v>07-Sept-2026, 2:37 pm</v>
+        <v>07-Sept-2026, 1:26 pm</v>
       </c>
       <c r="O2" t="str">
-        <v>Bhoomika Sankhla Resume.PNG</v>
+        <v>Hm</v>
       </c>
       <c r="P2" t="str">
-        <v/>
+        <v>Auto-scheduled via WhatsApp AI: "Yes" (In-Person)</v>
       </c>
     </row>
     <row r="3">
@@ -521,13 +521,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>Arjun Meena</v>
+        <v>Tanmay Jain</v>
       </c>
       <c r="C3" t="str">
-        <v>+918357977322</v>
+        <v>+919993297342</v>
       </c>
       <c r="D3" t="str">
-        <v>SEO &amp; AEO Expert</v>
+        <v>Digital Marketing Manager</v>
       </c>
       <c r="E3" t="str">
         <v>In-Person (Indore Office)</v>
@@ -539,13 +539,13 @@
         <v/>
       </c>
       <c r="H3" t="str">
-        <v>Interview Scheduled</v>
+        <v>Resume Received</v>
       </c>
       <c r="I3" t="str">
-        <v>08-Sept-2026, 11:00 am</v>
+        <v>Not Scheduled</v>
       </c>
       <c r="J3" t="str">
-        <v>Experienced (Full-Time)</v>
+        <v>6 years</v>
       </c>
       <c r="K3" t="str">
         <v>Indore</v>
@@ -557,13 +557,13 @@
         <v>NO</v>
       </c>
       <c r="N3" t="str">
-        <v>07-Sept-2026, 1:26 pm</v>
+        <v>07-Sept-2026, 11:48 am</v>
       </c>
       <c r="O3" t="str">
-        <v>Hm</v>
+        <v>6</v>
       </c>
       <c r="P3" t="str">
-        <v>Auto-scheduled via WhatsApp AI: "Yes" (In-Person)</v>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -571,10 +571,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>Tanmay Jain</v>
+        <v>Shyama's house of snacks</v>
       </c>
       <c r="C4" t="str">
-        <v>+919993297342</v>
+        <v>+917693884339</v>
       </c>
       <c r="D4" t="str">
         <v>Digital Marketing Manager</v>
@@ -589,13 +589,13 @@
         <v/>
       </c>
       <c r="H4" t="str">
-        <v>Resume Received</v>
+        <v>Interview Scheduled</v>
       </c>
       <c r="I4" t="str">
-        <v>Not Scheduled</v>
+        <v>05-Sept-2026, 11:00 am</v>
       </c>
       <c r="J4" t="str">
-        <v>6 years</v>
+        <v>Fresher (Paid Internship)</v>
       </c>
       <c r="K4" t="str">
         <v>Indore</v>
@@ -607,89 +607,90 @@
         <v>NO</v>
       </c>
       <c r="N4" t="str">
-        <v>07-Sept-2026, 11:48 am</v>
+        <v>04-Sept-2026, 2:28 pm</v>
       </c>
       <c r="O4" t="str">
-        <v>6</v>
+        <v>ok sir</v>
       </c>
       <c r="P4" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="5">
+        <v>Auto-scheduled via WhatsApp AI: "ok sir" (In-Person)</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>Shyama's house of snacks</v>
+        <v>BrandSetuDigital</v>
       </c>
       <c r="C5" t="str">
-        <v>+917693884339</v>
+        <v>+919669765911</v>
       </c>
       <c r="D5" t="str">
-        <v>Digital Marketing Manager</v>
+        <v>General Applicant</v>
       </c>
       <c r="E5" t="str">
         <v>In-Person (Indore Office)</v>
       </c>
       <c r="F5" t="str">
-        <v>YES</v>
+        <v>PENDING</v>
       </c>
       <c r="G5" t="str">
         <v/>
       </c>
       <c r="H5" t="str">
-        <v>Interview Scheduled</v>
+        <v>Resume Pending</v>
       </c>
       <c r="I5" t="str">
-        <v>05-Sept-2026, 11:00 am</v>
+        <v>Not Scheduled</v>
       </c>
       <c r="J5" t="str">
-        <v>Fresher (Paid Internship)</v>
+        <v/>
       </c>
       <c r="K5" t="str">
         <v>Indore</v>
       </c>
       <c r="L5" t="str">
-        <v>NO</v>
+        <v>YES</v>
       </c>
       <c r="M5" t="str">
         <v>NO</v>
       </c>
       <c r="N5" t="str">
-        <v>04-Sept-2026, 2:28 pm</v>
-      </c>
-      <c r="O5" t="str">
-        <v>ok sir</v>
+        <v>04-Sept-2026, 2:33 pm</v>
+      </c>
+      <c r="O5" t="str" xml:space="preserve">
+        <v xml:space="preserve">Thank you for contacting BrandSetu Digital! 
+Please let us know how we can help you.</v>
       </c>
       <c r="P5" t="str">
-        <v>Auto-scheduled via WhatsApp AI: "ok sir" (In-Person)</v>
-      </c>
-    </row>
-    <row r="6" xml:space="preserve">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>BrandSetuDigital</v>
+        <v>Mohit 🎬</v>
       </c>
       <c r="C6" t="str">
-        <v>+919669765911</v>
+        <v>+917470584339</v>
       </c>
       <c r="D6" t="str">
-        <v>General Applicant</v>
+        <v>Video Editor</v>
       </c>
       <c r="E6" t="str">
         <v>In-Person (Indore Office)</v>
       </c>
       <c r="F6" t="str">
-        <v>PENDING</v>
+        <v>YES</v>
       </c>
       <c r="G6" t="str">
         <v/>
       </c>
       <c r="H6" t="str">
-        <v>Resume Pending</v>
+        <v>Resume Received</v>
       </c>
       <c r="I6" t="str">
         <v>Not Scheduled</v>
@@ -701,20 +702,19 @@
         <v>Indore</v>
       </c>
       <c r="L6" t="str">
-        <v>YES</v>
+        <v>NO</v>
       </c>
       <c r="M6" t="str">
-        <v>NO</v>
+        <v>YES</v>
       </c>
       <c r="N6" t="str">
-        <v>04-Sept-2026, 2:33 pm</v>
-      </c>
-      <c r="O6" t="str" xml:space="preserve">
-        <v xml:space="preserve">Thank you for contacting BrandSetu Digital! 
-Please let us know how we can help you.</v>
+        <v>20-Aug-2026, 4:31 pm</v>
+      </c>
+      <c r="O6" t="str">
+        <v>Hi!</v>
       </c>
       <c r="P6" t="str">
-        <v/>
+        <v>Auto-scheduled via WhatsApp AI: "Tomorrow morning 12 pm"</v>
       </c>
     </row>
     <row r="7">
@@ -722,25 +722,25 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>Mohit 🎬</v>
+        <v>manshi</v>
       </c>
       <c r="C7" t="str">
-        <v>+917470584339</v>
+        <v>+917828966773</v>
       </c>
       <c r="D7" t="str">
-        <v>Video Editor</v>
+        <v>Digital Marketing Manager</v>
       </c>
       <c r="E7" t="str">
         <v>In-Person (Indore Office)</v>
       </c>
       <c r="F7" t="str">
-        <v>YES</v>
+        <v>PENDING</v>
       </c>
       <c r="G7" t="str">
         <v/>
       </c>
       <c r="H7" t="str">
-        <v>Resume Received</v>
+        <v>Resume Pending</v>
       </c>
       <c r="I7" t="str">
         <v>Not Scheduled</v>
@@ -752,19 +752,19 @@
         <v>Indore</v>
       </c>
       <c r="L7" t="str">
-        <v>NO</v>
+        <v>YES</v>
       </c>
       <c r="M7" t="str">
-        <v>YES</v>
+        <v>NO</v>
       </c>
       <c r="N7" t="str">
-        <v>20-Aug-2026, 4:31 pm</v>
+        <v>04-Sept-2026, 2:27 pm</v>
       </c>
       <c r="O7" t="str">
-        <v>Hi!</v>
+        <v>Manual Entry: Role Digital Marketing Manager, Portfolio: N/A</v>
       </c>
       <c r="P7" t="str">
-        <v>Auto-scheduled via WhatsApp AI: "Tomorrow morning 12 pm"</v>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -772,49 +772,49 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>manshi</v>
+        <v>Aabid</v>
       </c>
       <c r="C8" t="str">
-        <v>+917828966773</v>
+        <v>+917869724727</v>
       </c>
       <c r="D8" t="str">
-        <v>Digital Marketing Manager</v>
+        <v>AI Video Expert</v>
       </c>
       <c r="E8" t="str">
         <v>In-Person (Indore Office)</v>
       </c>
       <c r="F8" t="str">
-        <v>PENDING</v>
+        <v>YES</v>
       </c>
       <c r="G8" t="str">
         <v/>
       </c>
       <c r="H8" t="str">
-        <v>Resume Pending</v>
+        <v>Interview Scheduled</v>
       </c>
       <c r="I8" t="str">
-        <v>Not Scheduled</v>
+        <v>04-Sept-2026, 2:00 pm</v>
       </c>
       <c r="J8" t="str">
-        <v/>
+        <v>Experienced (Full-Time)</v>
       </c>
       <c r="K8" t="str">
         <v>Indore</v>
       </c>
       <c r="L8" t="str">
-        <v>YES</v>
+        <v>NO</v>
       </c>
       <c r="M8" t="str">
         <v>NO</v>
       </c>
       <c r="N8" t="str">
-        <v>04-Sept-2026, 2:27 pm</v>
+        <v>04-Sept-2026, 2:15 pm</v>
       </c>
       <c r="O8" t="str">
-        <v>Manual Entry: Role Digital Marketing Manager, Portfolio: N/A</v>
+        <v>Today 2 PM</v>
       </c>
       <c r="P8" t="str">
-        <v/>
+        <v>Auto-scheduled via WhatsApp AI: "Today 2 PM" (In-Person)</v>
       </c>
     </row>
     <row r="9">
@@ -822,49 +822,49 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>Aabid</v>
+        <v>Nancy Ajmera</v>
       </c>
       <c r="C9" t="str">
-        <v>+917869724727</v>
+        <v>+38899686625461</v>
       </c>
       <c r="D9" t="str">
-        <v>AI Video Expert</v>
+        <v>General Applicant</v>
       </c>
       <c r="E9" t="str">
         <v>In-Person (Indore Office)</v>
       </c>
       <c r="F9" t="str">
-        <v>YES</v>
+        <v>PENDING</v>
       </c>
       <c r="G9" t="str">
         <v/>
       </c>
       <c r="H9" t="str">
-        <v>Interview Scheduled</v>
+        <v>Applied</v>
       </c>
       <c r="I9" t="str">
-        <v>04-Sept-2026, 2:00 pm</v>
+        <v>Not Scheduled</v>
       </c>
       <c r="J9" t="str">
-        <v>Experienced (Full-Time)</v>
+        <v/>
       </c>
       <c r="K9" t="str">
         <v>Indore</v>
       </c>
       <c r="L9" t="str">
-        <v>NO</v>
+        <v>YES</v>
       </c>
       <c r="M9" t="str">
         <v>NO</v>
       </c>
       <c r="N9" t="str">
-        <v>04-Sept-2026, 2:15 pm</v>
+        <v>03-Sept-2026, 5:03 pm</v>
       </c>
       <c r="O9" t="str">
-        <v>Today 2 PM</v>
+        <v>Hello! Can I get more info on this?</v>
       </c>
       <c r="P9" t="str">
-        <v>Auto-scheduled via WhatsApp AI: "Today 2 PM" (In-Person)</v>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -872,49 +872,49 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>Nancy Ajmera</v>
+        <v>Unnat</v>
       </c>
       <c r="C10" t="str">
-        <v>+38899686625461</v>
+        <v>+278880866857060</v>
       </c>
       <c r="D10" t="str">
-        <v>General Applicant</v>
+        <v>Video Editor</v>
       </c>
       <c r="E10" t="str">
         <v>In-Person (Indore Office)</v>
       </c>
       <c r="F10" t="str">
-        <v>PENDING</v>
+        <v>YES</v>
       </c>
       <c r="G10" t="str">
-        <v/>
+        <v>https://corrra.com/@unnatportfolio</v>
       </c>
       <c r="H10" t="str">
-        <v>Applied</v>
+        <v>Interview Scheduled</v>
       </c>
       <c r="I10" t="str">
-        <v>Not Scheduled</v>
+        <v>04-Sept-2026, 4:00 pm</v>
       </c>
       <c r="J10" t="str">
-        <v/>
+        <v>Experienced (Full-Time)</v>
       </c>
       <c r="K10" t="str">
         <v>Indore</v>
       </c>
       <c r="L10" t="str">
-        <v>YES</v>
+        <v>NO</v>
       </c>
       <c r="M10" t="str">
-        <v>NO</v>
+        <v>YES</v>
       </c>
       <c r="N10" t="str">
-        <v>03-Sept-2026, 5:03 pm</v>
+        <v>03-Sept-2026, 3:58 pm</v>
       </c>
       <c r="O10" t="str">
-        <v>Hello! Can I get more info on this?</v>
+        <v>4 sep friday</v>
       </c>
       <c r="P10" t="str">
-        <v/>
+        <v>Auto-scheduled via WhatsApp AI: "4 sep friday"</v>
       </c>
     </row>
     <row r="11">
@@ -922,10 +922,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>Unnat</v>
+        <v>Arjun Meena</v>
       </c>
       <c r="C11" t="str">
-        <v>+278880866857060</v>
+        <v>+919329232025</v>
       </c>
       <c r="D11" t="str">
         <v>Video Editor</v>
@@ -937,16 +937,16 @@
         <v>YES</v>
       </c>
       <c r="G11" t="str">
-        <v>https://corrra.com/@unnatportfolio</v>
+        <v>https://drive.google.com/drive/folders/sample_portfolio</v>
       </c>
       <c r="H11" t="str">
         <v>Interview Scheduled</v>
       </c>
       <c r="I11" t="str">
-        <v>04-Sept-2026, 4:00 pm</v>
+        <v>04-Sept-2026, 2:00 pm</v>
       </c>
       <c r="J11" t="str">
-        <v>Experienced (Full-Time)</v>
+        <v>Fresher (Paid Internship)</v>
       </c>
       <c r="K11" t="str">
         <v>Indore</v>
@@ -958,13 +958,13 @@
         <v>YES</v>
       </c>
       <c r="N11" t="str">
-        <v>03-Sept-2026, 3:58 pm</v>
+        <v>03-Sept-2026, 3:35 pm</v>
       </c>
       <c r="O11" t="str">
-        <v>4 sep friday</v>
+        <v>Kal dopahar 2 baje</v>
       </c>
       <c r="P11" t="str">
-        <v>Auto-scheduled via WhatsApp AI: "4 sep friday"</v>
+        <v>Test auto schedule</v>
       </c>
     </row>
     <row r="12">
@@ -975,7 +975,7 @@
         <v>Arjun Meena</v>
       </c>
       <c r="C12" t="str">
-        <v>+919329232025</v>
+        <v>+114405211672638</v>
       </c>
       <c r="D12" t="str">
         <v>Video Editor</v>
@@ -987,13 +987,13 @@
         <v>YES</v>
       </c>
       <c r="G12" t="str">
-        <v>https://drive.google.com/drive/folders/sample_portfolio</v>
+        <v/>
       </c>
       <c r="H12" t="str">
         <v>Interview Scheduled</v>
       </c>
       <c r="I12" t="str">
-        <v>04-Sept-2026, 2:00 pm</v>
+        <v>03-Sept-2026, 5:00 pm</v>
       </c>
       <c r="J12" t="str">
         <v>Fresher (Paid Internship)</v>
@@ -1008,13 +1008,13 @@
         <v>YES</v>
       </c>
       <c r="N12" t="str">
-        <v>03-Sept-2026, 3:35 pm</v>
+        <v>03-Sept-2026, 2:29 pm</v>
       </c>
       <c r="O12" t="str">
-        <v>Kal dopahar 2 baje</v>
+        <v>Hiiii</v>
       </c>
       <c r="P12" t="str">
-        <v>Test auto schedule</v>
+        <v>Auto-scheduled via WhatsApp AI: "Today 5:3 mint pe mera interview resedule kr do"</v>
       </c>
     </row>
     <row r="13">
@@ -1022,10 +1022,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>Arjun Meena</v>
+        <v>manisha</v>
       </c>
       <c r="C13" t="str">
-        <v>+114405211672638</v>
+        <v>+917879010084</v>
       </c>
       <c r="D13" t="str">
         <v>Video Editor</v>
@@ -1034,92 +1034,42 @@
         <v>In-Person (Indore Office)</v>
       </c>
       <c r="F13" t="str">
-        <v>YES</v>
+        <v>PENDING</v>
       </c>
       <c r="G13" t="str">
         <v/>
       </c>
       <c r="H13" t="str">
-        <v>Interview Scheduled</v>
+        <v>Resume Pending</v>
       </c>
       <c r="I13" t="str">
-        <v>03-Sept-2026, 5:00 pm</v>
+        <v>Not Scheduled</v>
       </c>
       <c r="J13" t="str">
-        <v>Fresher (Paid Internship)</v>
+        <v/>
       </c>
       <c r="K13" t="str">
         <v>Indore</v>
       </c>
       <c r="L13" t="str">
-        <v>NO</v>
+        <v>YES</v>
       </c>
       <c r="M13" t="str">
-        <v>YES</v>
+        <v>NO</v>
       </c>
       <c r="N13" t="str">
-        <v>03-Sept-2026, 2:29 pm</v>
+        <v>20-Aug-2026, 3:49 pm</v>
       </c>
       <c r="O13" t="str">
-        <v>Hiiii</v>
+        <v>Manual Entry: Role Video Editor, Portfolio: N/A</v>
       </c>
       <c r="P13" t="str">
-        <v>Auto-scheduled via WhatsApp AI: "Today 5:3 mint pe mera interview resedule kr do"</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="str">
-        <v>manisha</v>
-      </c>
-      <c r="C14" t="str">
-        <v>+917879010084</v>
-      </c>
-      <c r="D14" t="str">
-        <v>Video Editor</v>
-      </c>
-      <c r="E14" t="str">
-        <v>In-Person (Indore Office)</v>
-      </c>
-      <c r="F14" t="str">
-        <v>PENDING</v>
-      </c>
-      <c r="G14" t="str">
-        <v/>
-      </c>
-      <c r="H14" t="str">
-        <v>Resume Pending</v>
-      </c>
-      <c r="I14" t="str">
-        <v>Not Scheduled</v>
-      </c>
-      <c r="J14" t="str">
-        <v/>
-      </c>
-      <c r="K14" t="str">
-        <v>Indore</v>
-      </c>
-      <c r="L14" t="str">
-        <v>YES</v>
-      </c>
-      <c r="M14" t="str">
-        <v>NO</v>
-      </c>
-      <c r="N14" t="str">
-        <v>20-Aug-2026, 3:49 pm</v>
-      </c>
-      <c r="O14" t="str">
-        <v>Manual Entry: Role Video Editor, Portfolio: N/A</v>
-      </c>
-      <c r="P14" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>